<commit_message>
Auto update Pengadaan 2026-10-20 12:43:22
</commit_message>
<xml_diff>
--- a/output/tepra/2026/Tepra Kobar_Progres PBJ tahun 2026 (2026-10-20).xlsx
+++ b/output/tepra/2026/Tepra Kobar_Progres PBJ tahun 2026 (2026-10-20).xlsx
@@ -1020,27 +1020,35 @@
           <t>DINAS PEKERJAAN UMUM DAN PENATAAN RUANG - 1.03.0.00.0.00.01.0000</t>
         </is>
       </c>
-      <c r="C17" s="4" t="n">
-        <v>1</v>
+      <c r="C17" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="D17" s="6" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="E17" s="4" t="n">
-        <v>1</v>
+      <c r="E17" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="F17" s="6" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="G17" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="H17" s="11" t="n">
-        <v>1796500000</v>
+      <c r="G17" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H17" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="I17" s="6" t="inlineStr">
         <is>
@@ -1162,27 +1170,35 @@
           <t>DINAS PERINDUSTRIAN, PERDAGANGAN, KOPERASI, USAHA KECIL DAN MENENGAH - 2.17.3.30.3.31.01.0000</t>
         </is>
       </c>
-      <c r="C20" s="7" t="n">
-        <v>3</v>
+      <c r="C20" s="10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="D20" s="10" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="E20" s="7" t="n">
-        <v>3</v>
+      <c r="E20" s="10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="F20" s="10" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="G20" s="7" t="n">
-        <v>3</v>
-      </c>
-      <c r="H20" s="9" t="n">
-        <v>3839600910</v>
+      <c r="G20" s="10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H20" s="10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="I20" s="10" t="inlineStr">
         <is>
@@ -1308,13 +1324,13 @@
         <v>95</v>
       </c>
       <c r="D23" s="11" t="n">
-        <v>1153832942</v>
+        <v>1151066942</v>
       </c>
       <c r="E23" s="4" t="n">
         <v>5</v>
       </c>
       <c r="F23" s="11" t="n">
-        <v>62227794</v>
+        <v>59461794</v>
       </c>
       <c r="G23" s="4" t="n">
         <v>5</v>
@@ -1339,22 +1355,22 @@
         </is>
       </c>
       <c r="C24" s="7" t="n">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D24" s="9" t="n">
-        <v>403884747</v>
+        <v>414639535</v>
       </c>
       <c r="E24" s="7" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F24" s="9" t="n">
-        <v>74152766</v>
+        <v>84907554</v>
       </c>
       <c r="G24" s="7" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="H24" s="9" t="n">
-        <v>128214258</v>
+        <v>78869208</v>
       </c>
       <c r="I24" s="7" t="n">
         <v>62</v>
@@ -1373,22 +1389,22 @@
         </is>
       </c>
       <c r="C25" s="4" t="n">
-        <v>130</v>
+        <v>105</v>
       </c>
       <c r="D25" s="11" t="n">
-        <v>762684358</v>
+        <v>753671912</v>
       </c>
       <c r="E25" s="4" t="n">
-        <v>38</v>
+        <v>13</v>
       </c>
       <c r="F25" s="11" t="n">
-        <v>146596290</v>
+        <v>137583844</v>
       </c>
       <c r="G25" s="4" t="n">
-        <v>38</v>
+        <v>13</v>
       </c>
       <c r="H25" s="11" t="n">
-        <v>1345382085</v>
+        <v>116218702</v>
       </c>
       <c r="I25" s="4" t="n">
         <v>92</v>
@@ -1407,22 +1423,22 @@
         </is>
       </c>
       <c r="C26" s="7" t="n">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D26" s="9" t="n">
         <v>497942073</v>
       </c>
       <c r="E26" s="7" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F26" s="9" t="n">
         <v>338217900</v>
       </c>
       <c r="G26" s="7" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H26" s="9" t="n">
-        <v>3037348900</v>
+        <v>338050900</v>
       </c>
       <c r="I26" s="7" t="n">
         <v>22</v>
@@ -1478,13 +1494,13 @@
         <v>100</v>
       </c>
       <c r="D28" s="9" t="n">
-        <v>890948817</v>
+        <v>900575817</v>
       </c>
       <c r="E28" s="7" t="n">
         <v>1</v>
       </c>
       <c r="F28" s="9" t="n">
-        <v>28881000</v>
+        <v>38508000</v>
       </c>
       <c r="G28" s="7" t="n">
         <v>1</v>
@@ -1512,13 +1528,13 @@
         <v>181</v>
       </c>
       <c r="D29" s="11" t="n">
-        <v>2495843490</v>
+        <v>2505347643</v>
       </c>
       <c r="E29" s="4" t="n">
         <v>54</v>
       </c>
       <c r="F29" s="11" t="n">
-        <v>1126736515</v>
+        <v>1136240668</v>
       </c>
       <c r="G29" s="4" t="n">
         <v>54</v>
@@ -1543,22 +1559,22 @@
         </is>
       </c>
       <c r="C30" s="7" t="n">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D30" s="9" t="n">
         <v>367878502</v>
       </c>
       <c r="E30" s="7" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F30" s="9" t="n">
         <v>80601092</v>
       </c>
       <c r="G30" s="7" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="H30" s="9" t="n">
-        <v>227435607</v>
+        <v>77435607</v>
       </c>
       <c r="I30" s="7" t="n">
         <v>48</v>
@@ -1580,13 +1596,13 @@
         <v>52</v>
       </c>
       <c r="D31" s="11" t="n">
-        <v>283157746</v>
+        <v>283301771</v>
       </c>
       <c r="E31" s="4" t="n">
         <v>5</v>
       </c>
       <c r="F31" s="11" t="n">
-        <v>30118025</v>
+        <v>30262050</v>
       </c>
       <c r="G31" s="4" t="n">
         <v>5</v>
@@ -1614,13 +1630,13 @@
         <v>122</v>
       </c>
       <c r="D32" s="9" t="n">
-        <v>764274671</v>
+        <v>767894130</v>
       </c>
       <c r="E32" s="7" t="n">
         <v>6</v>
       </c>
       <c r="F32" s="9" t="n">
-        <v>103722907</v>
+        <v>107342366</v>
       </c>
       <c r="G32" s="7" t="n">
         <v>6</v>
@@ -1648,13 +1664,13 @@
         <v>44</v>
       </c>
       <c r="D33" s="11" t="n">
-        <v>278301799</v>
+        <v>366634933</v>
       </c>
       <c r="E33" s="4" t="n">
         <v>5</v>
       </c>
       <c r="F33" s="11" t="n">
-        <v>20641550</v>
+        <v>108974684</v>
       </c>
       <c r="G33" s="4" t="n">
         <v>5</v>
@@ -1716,13 +1732,13 @@
         <v>66</v>
       </c>
       <c r="D35" s="11" t="n">
-        <v>463836830</v>
+        <v>463972148</v>
       </c>
       <c r="E35" s="4" t="n">
         <v>6</v>
       </c>
       <c r="F35" s="11" t="n">
-        <v>93231105</v>
+        <v>93366423</v>
       </c>
       <c r="G35" s="4" t="n">
         <v>6</v>
@@ -1781,22 +1797,22 @@
         </is>
       </c>
       <c r="C37" s="4" t="n">
-        <v>108</v>
+        <v>100</v>
       </c>
       <c r="D37" s="11" t="n">
-        <v>844312891</v>
+        <v>1224904791</v>
       </c>
       <c r="E37" s="4" t="n">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="F37" s="11" t="n">
-        <v>81094602</v>
+        <v>461686502</v>
       </c>
       <c r="G37" s="4" t="n">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="H37" s="11" t="n">
-        <v>1530548790</v>
+        <v>451166160</v>
       </c>
       <c r="I37" s="4" t="n">
         <v>84</v>
@@ -1818,13 +1834,13 @@
         <v>97</v>
       </c>
       <c r="D38" s="9" t="n">
-        <v>382731831</v>
+        <v>384332451</v>
       </c>
       <c r="E38" s="7" t="n">
         <v>11</v>
       </c>
       <c r="F38" s="9" t="n">
-        <v>85740718</v>
+        <v>87341338</v>
       </c>
       <c r="G38" s="7" t="n">
         <v>11</v>
@@ -1849,22 +1865,22 @@
         </is>
       </c>
       <c r="C39" s="4" t="n">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D39" s="11" t="n">
-        <v>1287902678</v>
+        <v>1313432678</v>
       </c>
       <c r="E39" s="4" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F39" s="11" t="n">
-        <v>352528156</v>
+        <v>378058156</v>
       </c>
       <c r="G39" s="4" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="H39" s="11" t="n">
-        <v>414800436</v>
+        <v>374723886</v>
       </c>
       <c r="I39" s="4" t="n">
         <v>87</v>
@@ -1988,13 +2004,13 @@
         <v>50</v>
       </c>
       <c r="D43" s="11" t="n">
-        <v>727698127</v>
+        <v>708077545</v>
       </c>
       <c r="E43" s="4" t="n">
         <v>3</v>
       </c>
       <c r="F43" s="11" t="n">
-        <v>54570486</v>
+        <v>34949904</v>
       </c>
       <c r="G43" s="4" t="n">
         <v>3</v>
@@ -2019,22 +2035,22 @@
         </is>
       </c>
       <c r="C44" s="7" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D44" s="9" t="n">
         <v>282819298</v>
       </c>
       <c r="E44" s="7" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F44" s="9" t="n">
         <v>151137140</v>
       </c>
       <c r="G44" s="7" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H44" s="9" t="n">
-        <v>83626512</v>
+        <v>72726534</v>
       </c>
       <c r="I44" s="7" t="n">
         <v>15</v>
@@ -2103,22 +2119,22 @@
         </is>
       </c>
       <c r="C46" s="7" t="n">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="D46" s="9" t="n">
-        <v>1174813471</v>
+        <v>1126161061</v>
       </c>
       <c r="E46" s="7" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="F46" s="9" t="n">
-        <v>173625311</v>
+        <v>124972901</v>
       </c>
       <c r="G46" s="7" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="H46" s="9" t="n">
-        <v>318350703</v>
+        <v>121983128</v>
       </c>
       <c r="I46" s="7" t="n">
         <v>169</v>
@@ -2224,13 +2240,13 @@
         <v>102</v>
       </c>
       <c r="D49" s="11" t="n">
-        <v>606361476</v>
+        <v>608286476</v>
       </c>
       <c r="E49" s="4" t="n">
         <v>15</v>
       </c>
       <c r="F49" s="11" t="n">
-        <v>203015123</v>
+        <v>204940123</v>
       </c>
       <c r="G49" s="4" t="n">
         <v>15</v>
@@ -2339,24 +2355,30 @@
         </is>
       </c>
       <c r="C52" s="7" t="n">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="D52" s="9" t="n">
         <v>111669795</v>
       </c>
-      <c r="E52" s="7" t="n">
-        <v>3</v>
+      <c r="E52" s="10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="F52" s="10" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="G52" s="7" t="n">
-        <v>3</v>
-      </c>
-      <c r="H52" s="9" t="n">
-        <v>68020787</v>
+      <c r="G52" s="10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H52" s="10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="I52" s="7" t="n">
         <v>14</v>
@@ -3126,13 +3148,13 @@
         <v>41</v>
       </c>
       <c r="D71" s="11" t="n">
-        <v>323431257</v>
+        <v>330321582</v>
       </c>
       <c r="E71" s="4" t="n">
         <v>2</v>
       </c>
       <c r="F71" s="11" t="n">
-        <v>28826575</v>
+        <v>35716900</v>
       </c>
       <c r="G71" s="4" t="n">
         <v>2</v>
@@ -3157,22 +3179,22 @@
         </is>
       </c>
       <c r="C72" s="7" t="n">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="D72" s="9" t="n">
         <v>637283463</v>
       </c>
       <c r="E72" s="7" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="F72" s="9" t="n">
         <v>108000000</v>
       </c>
       <c r="G72" s="7" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="H72" s="9" t="n">
-        <v>2359971000</v>
+        <v>158730000</v>
       </c>
       <c r="I72" s="7" t="n">
         <v>29</v>
@@ -3278,7 +3300,7 @@
         <v>113</v>
       </c>
       <c r="D75" s="11" t="n">
-        <v>1398754546</v>
+        <v>1433154546</v>
       </c>
       <c r="E75" s="4" t="n">
         <v>18</v>
@@ -3296,7 +3318,7 @@
         <v>95</v>
       </c>
       <c r="J75" s="11" t="n">
-        <v>978880360</v>
+        <v>1013280360</v>
       </c>
     </row>
     <row r="76" ht="45" customHeight="1">
@@ -3309,22 +3331,22 @@
         </is>
       </c>
       <c r="C76" s="7" t="n">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="D76" s="9" t="n">
-        <v>1105997520</v>
+        <v>1183031520</v>
       </c>
       <c r="E76" s="7" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="F76" s="9" t="n">
-        <v>136951114</v>
+        <v>213985114</v>
       </c>
       <c r="G76" s="7" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="H76" s="9" t="n">
-        <v>351515407</v>
+        <v>202015407</v>
       </c>
       <c r="I76" s="7" t="n">
         <v>111</v>
@@ -3341,28 +3363,28 @@
         </is>
       </c>
       <c r="C77" s="12" t="n">
-        <v>4047</v>
+        <v>3996</v>
       </c>
       <c r="D77" s="13" t="n">
-        <v>33723764043</v>
+        <v>34293802327</v>
       </c>
       <c r="E77" s="12" t="n">
-        <v>467</v>
+        <v>416</v>
       </c>
       <c r="F77" s="13" t="n">
-        <v>6209464834</v>
+        <v>6745103118</v>
       </c>
       <c r="G77" s="12" t="n">
-        <v>467</v>
+        <v>416</v>
       </c>
       <c r="H77" s="13" t="n">
-        <v>19844451365.6</v>
+        <v>6335055502.6</v>
       </c>
       <c r="I77" s="12" t="n">
         <v>3580</v>
       </c>
       <c r="J77" s="13" t="n">
-        <v>27514299209</v>
+        <v>27548699209</v>
       </c>
     </row>
   </sheetData>
@@ -3783,13 +3805,13 @@
         <v>5</v>
       </c>
       <c r="D11" s="11" t="n">
-        <v>413165330</v>
+        <v>428765330</v>
       </c>
       <c r="E11" s="4" t="n">
         <v>3</v>
       </c>
       <c r="F11" s="11" t="n">
-        <v>261110330</v>
+        <v>276710330</v>
       </c>
       <c r="G11" s="4" t="n">
         <v>3</v>
@@ -4219,29 +4241,45 @@
           <t>DINAS PERHUBUNGAN - 2.15.0.00.0.00.01.0000</t>
         </is>
       </c>
-      <c r="C19" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="D19" s="11" t="n">
-        <v>199078500</v>
-      </c>
-      <c r="E19" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="F19" s="11" t="n">
-        <v>199078500</v>
-      </c>
-      <c r="G19" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="H19" s="11" t="n">
-        <v>199078500</v>
-      </c>
-      <c r="I19" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="J19" s="11" t="n">
-        <v>199078500</v>
+      <c r="C19" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D19" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E19" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F19" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G19" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H19" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I19" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J19" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="K19" s="6" t="inlineStr">
         <is>
@@ -4273,45 +4311,29 @@
           <t>DINAS PERINDUSTRIAN, PERDAGANGAN, KOPERASI, USAHA KECIL DAN MENENGAH - 2.17.3.30.3.31.01.0000</t>
         </is>
       </c>
-      <c r="C20" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D20" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E20" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F20" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G20" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H20" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I20" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J20" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="C20" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D20" s="9" t="n">
+        <v>112000000</v>
+      </c>
+      <c r="E20" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F20" s="9" t="n">
+        <v>112000000</v>
+      </c>
+      <c r="G20" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="H20" s="9" t="n">
+        <v>111200910</v>
+      </c>
+      <c r="I20" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="J20" s="9" t="n">
+        <v>111200910</v>
       </c>
       <c r="K20" s="10" t="inlineStr">
         <is>
@@ -4534,50 +4556,34 @@
         </is>
       </c>
       <c r="C24" s="7" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D24" s="9" t="n">
-        <v>268961631</v>
-      </c>
-      <c r="E24" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F24" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G24" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H24" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I24" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J24" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K24" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L24" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+        <v>323734637</v>
+      </c>
+      <c r="E24" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F24" s="9" t="n">
+        <v>54773006</v>
+      </c>
+      <c r="G24" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="H24" s="9" t="n">
+        <v>49345050</v>
+      </c>
+      <c r="I24" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="J24" s="9" t="n">
+        <v>49345050</v>
+      </c>
+      <c r="K24" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="L24" s="9" t="n">
+        <v>49345050</v>
       </c>
       <c r="M24" s="7" t="n">
         <v>3</v>
@@ -4596,28 +4602,28 @@
         </is>
       </c>
       <c r="C25" s="4" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="D25" s="11" t="n">
-        <v>1368248170</v>
+        <v>1588904113</v>
       </c>
       <c r="E25" s="4" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="F25" s="11" t="n">
-        <v>1004886595</v>
+        <v>1225542538</v>
       </c>
       <c r="G25" s="4" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="H25" s="11" t="n">
-        <v>852531955</v>
+        <v>896262562</v>
       </c>
       <c r="I25" s="4" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="J25" s="11" t="n">
-        <v>852531955</v>
+        <v>896262562</v>
       </c>
       <c r="K25" s="4" t="n">
         <v>4</v>
@@ -4842,28 +4848,28 @@
         </is>
       </c>
       <c r="C30" s="7" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D30" s="9" t="n">
-        <v>388286000</v>
+        <v>538286000</v>
       </c>
       <c r="E30" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F30" s="9" t="n">
-        <v>138750000</v>
+        <v>288750000</v>
       </c>
       <c r="G30" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H30" s="9" t="n">
-        <v>138306000</v>
+        <v>288306000</v>
       </c>
       <c r="I30" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J30" s="9" t="n">
-        <v>138306000</v>
+        <v>288306000</v>
       </c>
       <c r="K30" s="10" t="inlineStr">
         <is>
@@ -4895,13 +4901,13 @@
         <v>7</v>
       </c>
       <c r="D31" s="11" t="n">
-        <v>490395090</v>
+        <v>477133090</v>
       </c>
       <c r="E31" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F31" s="11" t="n">
-        <v>79572000</v>
+        <v>66310000</v>
       </c>
       <c r="G31" s="4" t="n">
         <v>1</v>
@@ -5095,13 +5101,13 @@
         <v>13</v>
       </c>
       <c r="D35" s="11" t="n">
-        <v>1667542131</v>
+        <v>1694840343</v>
       </c>
       <c r="E35" s="4" t="n">
         <v>7</v>
       </c>
       <c r="F35" s="11" t="n">
-        <v>885723156</v>
+        <v>913021368</v>
       </c>
       <c r="G35" s="4" t="n">
         <v>7</v>
@@ -5192,34 +5198,34 @@
         </is>
       </c>
       <c r="C37" s="4" t="n">
-        <v>26</v>
+        <v>33</v>
       </c>
       <c r="D37" s="11" t="n">
-        <v>2613177050</v>
+        <v>3261325550</v>
       </c>
       <c r="E37" s="4" t="n">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="F37" s="11" t="n">
-        <v>1376941951</v>
+        <v>2025090451</v>
       </c>
       <c r="G37" s="4" t="n">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="H37" s="11" t="n">
-        <v>1333233523</v>
+        <v>1975819523</v>
       </c>
       <c r="I37" s="4" t="n">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="J37" s="11" t="n">
-        <v>1123727573</v>
+        <v>1581713573</v>
       </c>
       <c r="K37" s="4" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="L37" s="11" t="n">
-        <v>275128133</v>
+        <v>622336133</v>
       </c>
       <c r="M37" s="4" t="n">
         <v>13</v>
@@ -5300,28 +5306,28 @@
         </is>
       </c>
       <c r="C39" s="4" t="n">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="D39" s="11" t="n">
-        <v>4127193593</v>
+        <v>4380291888</v>
       </c>
       <c r="E39" s="4" t="n">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="F39" s="11" t="n">
-        <v>2516286291</v>
+        <v>2769384586</v>
       </c>
       <c r="G39" s="4" t="n">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="H39" s="11" t="n">
-        <v>2483413043</v>
+        <v>2708459593</v>
       </c>
       <c r="I39" s="4" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="J39" s="11" t="n">
-        <v>970364883</v>
+        <v>1155334883</v>
       </c>
       <c r="K39" s="4" t="n">
         <v>1</v>
@@ -5574,28 +5580,28 @@
         </is>
       </c>
       <c r="C44" s="7" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D44" s="9" t="n">
-        <v>523391100</v>
+        <v>595373450</v>
       </c>
       <c r="E44" s="7" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F44" s="9" t="n">
-        <v>345935300</v>
+        <v>417917650</v>
       </c>
       <c r="G44" s="7" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H44" s="9" t="n">
-        <v>187868022</v>
+        <v>198768000</v>
       </c>
       <c r="I44" s="7" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J44" s="9" t="n">
-        <v>187868022</v>
+        <v>198768000</v>
       </c>
       <c r="K44" s="7" t="n">
         <v>1</v>
@@ -5690,28 +5696,28 @@
         </is>
       </c>
       <c r="C46" s="7" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="D46" s="9" t="n">
-        <v>716222170</v>
+        <v>932380105</v>
       </c>
       <c r="E46" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="F46" s="9" t="n">
+        <v>471330601</v>
+      </c>
+      <c r="G46" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="H46" s="9" t="n">
+        <v>448555830</v>
+      </c>
+      <c r="I46" s="7" t="n">
         <v>4</v>
       </c>
-      <c r="F46" s="9" t="n">
-        <v>255172666</v>
-      </c>
-      <c r="G46" s="7" t="n">
-        <v>4</v>
-      </c>
-      <c r="H46" s="9" t="n">
-        <v>252188255</v>
-      </c>
-      <c r="I46" s="7" t="n">
-        <v>2</v>
-      </c>
       <c r="J46" s="9" t="n">
-        <v>113248255</v>
+        <v>309615830</v>
       </c>
       <c r="K46" s="10" t="inlineStr">
         <is>
@@ -6034,40 +6040,28 @@
         </is>
       </c>
       <c r="C52" s="7" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="D52" s="9" t="n">
-        <v>319983894</v>
-      </c>
-      <c r="E52" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F52" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G52" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H52" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I52" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J52" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+        <v>660566066</v>
+      </c>
+      <c r="E52" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="F52" s="9" t="n">
+        <v>340582172</v>
+      </c>
+      <c r="G52" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="H52" s="9" t="n">
+        <v>68020787</v>
+      </c>
+      <c r="I52" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="J52" s="9" t="n">
+        <v>68020787</v>
       </c>
       <c r="K52" s="10" t="inlineStr">
         <is>
@@ -7219,13 +7213,13 @@
         <v>3</v>
       </c>
       <c r="D71" s="11" t="n">
-        <v>392285593</v>
+        <v>423288615</v>
       </c>
       <c r="E71" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F71" s="11" t="n">
-        <v>115814581</v>
+        <v>146817603</v>
       </c>
       <c r="G71" s="4" t="n">
         <v>1</v>
@@ -7534,34 +7528,34 @@
         </is>
       </c>
       <c r="C77" s="12" t="n">
-        <v>861</v>
+        <v>880</v>
       </c>
       <c r="D77" s="13" t="n">
-        <v>102251454434</v>
+        <v>104180413369</v>
       </c>
       <c r="E77" s="12" t="n">
-        <v>502</v>
+        <v>521</v>
       </c>
       <c r="F77" s="13" t="n">
-        <v>63756505724</v>
+        <v>65685464659</v>
       </c>
       <c r="G77" s="12" t="n">
-        <v>502</v>
+        <v>521</v>
       </c>
       <c r="H77" s="13" t="n">
-        <v>62787645930.41</v>
+        <v>64085764887.41</v>
       </c>
       <c r="I77" s="12" t="n">
-        <v>290</v>
+        <v>307</v>
       </c>
       <c r="J77" s="13" t="n">
-        <v>36631038276.02</v>
+        <v>37704480683.02</v>
       </c>
       <c r="K77" s="12" t="n">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="L77" s="13" t="n">
-        <v>807344298</v>
+        <v>1203897348</v>
       </c>
       <c r="M77" s="12" t="n">
         <v>359</v>
@@ -8369,28 +8363,28 @@
         </is>
       </c>
       <c r="C17" s="4" t="n">
+        <v>23</v>
+      </c>
+      <c r="D17" s="11" t="n">
+        <v>26735477939</v>
+      </c>
+      <c r="E17" s="4" t="n">
+        <v>23</v>
+      </c>
+      <c r="F17" s="11" t="n">
+        <v>26735477939</v>
+      </c>
+      <c r="G17" s="4" t="n">
+        <v>23</v>
+      </c>
+      <c r="H17" s="11" t="n">
+        <v>26394591741</v>
+      </c>
+      <c r="I17" s="4" t="n">
         <v>22</v>
       </c>
-      <c r="D17" s="11" t="n">
-        <v>25286544212</v>
-      </c>
-      <c r="E17" s="4" t="n">
-        <v>22</v>
-      </c>
-      <c r="F17" s="11" t="n">
-        <v>25286544212</v>
-      </c>
-      <c r="G17" s="4" t="n">
-        <v>22</v>
-      </c>
-      <c r="H17" s="11" t="n">
-        <v>24598091741</v>
-      </c>
-      <c r="I17" s="4" t="n">
-        <v>21</v>
-      </c>
       <c r="J17" s="11" t="n">
-        <v>24598091741</v>
+        <v>26394591741</v>
       </c>
       <c r="K17" s="6" t="inlineStr">
         <is>
@@ -8476,45 +8470,29 @@
           <t>DINAS PERHUBUNGAN - 2.15.0.00.0.00.01.0000</t>
         </is>
       </c>
-      <c r="C19" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D19" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E19" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F19" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G19" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H19" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I19" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J19" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="C19" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="D19" s="11" t="n">
+        <v>201600000</v>
+      </c>
+      <c r="E19" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F19" s="11" t="n">
+        <v>201600000</v>
+      </c>
+      <c r="G19" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H19" s="11" t="n">
+        <v>199078500</v>
+      </c>
+      <c r="I19" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="J19" s="11" t="n">
+        <v>199078500</v>
       </c>
       <c r="K19" s="6" t="inlineStr">
         <is>
@@ -8546,45 +8524,29 @@
           <t>DINAS PERINDUSTRIAN, PERDAGANGAN, KOPERASI, USAHA KECIL DAN MENENGAH - 2.17.3.30.3.31.01.0000</t>
         </is>
       </c>
-      <c r="C20" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D20" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E20" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F20" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G20" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H20" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I20" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J20" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="C20" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D20" s="9" t="n">
+        <v>1090890000</v>
+      </c>
+      <c r="E20" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F20" s="9" t="n">
+        <v>1090890000</v>
+      </c>
+      <c r="G20" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="H20" s="9" t="n">
+        <v>1081900000</v>
+      </c>
+      <c r="I20" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="J20" s="9" t="n">
+        <v>1081900000</v>
       </c>
       <c r="K20" s="10" t="inlineStr">
         <is>
@@ -8620,13 +8582,13 @@
         <v>1</v>
       </c>
       <c r="D21" s="11" t="n">
-        <v>634957185</v>
+        <v>1269914370</v>
       </c>
       <c r="E21" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F21" s="11" t="n">
-        <v>634957185</v>
+        <v>1269914370</v>
       </c>
       <c r="G21" s="4" t="n">
         <v>1</v>
@@ -8674,7 +8636,7 @@
         <v>1</v>
       </c>
       <c r="D22" s="9" t="n">
-        <v>272000000</v>
+        <v>277500000</v>
       </c>
       <c r="E22" s="10" t="inlineStr">
         <is>
@@ -8720,7 +8682,7 @@
         <v>1</v>
       </c>
       <c r="N22" s="9" t="n">
-        <v>272000000</v>
+        <v>277500000</v>
       </c>
     </row>
     <row r="23" ht="45" customHeight="1">
@@ -8853,34 +8815,34 @@
         </is>
       </c>
       <c r="C25" s="4" t="n">
-        <v>10</v>
+        <v>33</v>
       </c>
       <c r="D25" s="11" t="n">
-        <v>5612329186</v>
+        <v>47963801011</v>
       </c>
       <c r="E25" s="4" t="n">
-        <v>9</v>
+        <v>32</v>
       </c>
       <c r="F25" s="11" t="n">
-        <v>5281245056</v>
+        <v>47632716881</v>
       </c>
       <c r="G25" s="4" t="n">
-        <v>9</v>
+        <v>32</v>
       </c>
       <c r="H25" s="11" t="n">
-        <v>2971571974</v>
+        <v>4157004750</v>
       </c>
       <c r="I25" s="4" t="n">
-        <v>9</v>
+        <v>32</v>
       </c>
       <c r="J25" s="11" t="n">
-        <v>2971571974</v>
+        <v>4157004750</v>
       </c>
       <c r="K25" s="4" t="n">
-        <v>6</v>
+        <v>27</v>
       </c>
       <c r="L25" s="11" t="n">
-        <v>1854621974</v>
+        <v>2945468782</v>
       </c>
       <c r="M25" s="4" t="n">
         <v>1</v>
@@ -9537,38 +9499,34 @@
         </is>
       </c>
       <c r="C37" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D37" s="11" t="n">
-        <v>5061390898</v>
+        <v>5934990898</v>
       </c>
       <c r="E37" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F37" s="11" t="n">
-        <v>2073094000</v>
+        <v>2946694000</v>
       </c>
       <c r="G37" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H37" s="11" t="n">
-        <v>2073094000</v>
+        <v>2509890630</v>
       </c>
       <c r="I37" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J37" s="11" t="n">
-        <v>2073094000</v>
-      </c>
-      <c r="K37" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L37" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+        <v>2509890630</v>
+      </c>
+      <c r="K37" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="L37" s="11" t="n">
+        <v>436796630</v>
       </c>
       <c r="M37" s="4" t="n">
         <v>4</v>
@@ -9657,28 +9615,28 @@
         </is>
       </c>
       <c r="C39" s="4" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D39" s="11" t="n">
-        <v>3962367980</v>
+        <v>3813601480</v>
       </c>
       <c r="E39" s="4" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F39" s="11" t="n">
-        <v>3162607980</v>
+        <v>3013841480</v>
       </c>
       <c r="G39" s="4" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="H39" s="11" t="n">
-        <v>2481708818</v>
+        <v>2296738818</v>
       </c>
       <c r="I39" s="4" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="J39" s="11" t="n">
-        <v>2481708818</v>
+        <v>2296738818</v>
       </c>
       <c r="K39" s="6" t="inlineStr">
         <is>
@@ -9884,13 +9842,13 @@
         <v>1</v>
       </c>
       <c r="D43" s="11" t="n">
-        <v>328338000</v>
+        <v>346000000</v>
       </c>
       <c r="E43" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F43" s="11" t="n">
-        <v>328338000</v>
+        <v>346000000</v>
       </c>
       <c r="G43" s="4" t="n">
         <v>1</v>
@@ -11811,28 +11769,28 @@
         </is>
       </c>
       <c r="C72" s="7" t="n">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="D72" s="9" t="n">
-        <v>7792798637</v>
+        <v>14398798637</v>
       </c>
       <c r="E72" s="7" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="F72" s="9" t="n">
-        <v>1448692000</v>
+        <v>8054692000</v>
       </c>
       <c r="G72" s="7" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="H72" s="9" t="n">
-        <v>607099212</v>
+        <v>2808340212</v>
       </c>
       <c r="I72" s="7" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="J72" s="9" t="n">
-        <v>607099212</v>
+        <v>2808340212</v>
       </c>
       <c r="K72" s="7" t="n">
         <v>2</v>
@@ -12023,28 +11981,28 @@
         </is>
       </c>
       <c r="C76" s="7" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D76" s="9" t="n">
-        <v>5020137400</v>
+        <v>5370137400</v>
       </c>
       <c r="E76" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="F76" s="9" t="n">
+        <v>3294207800</v>
+      </c>
+      <c r="G76" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="H76" s="9" t="n">
+        <v>2207941500</v>
+      </c>
+      <c r="I76" s="7" t="n">
         <v>4</v>
       </c>
-      <c r="F76" s="9" t="n">
-        <v>2944207800</v>
-      </c>
-      <c r="G76" s="7" t="n">
-        <v>4</v>
-      </c>
-      <c r="H76" s="9" t="n">
-        <v>2058441500</v>
-      </c>
-      <c r="I76" s="7" t="n">
-        <v>3</v>
-      </c>
       <c r="J76" s="9" t="n">
-        <v>2058441500</v>
+        <v>2207941500</v>
       </c>
       <c r="K76" s="10" t="inlineStr">
         <is>
@@ -12071,40 +12029,40 @@
         </is>
       </c>
       <c r="C77" s="12" t="n">
-        <v>209</v>
+        <v>239</v>
       </c>
       <c r="D77" s="13" t="n">
-        <v>129201730478</v>
+        <v>182633578715</v>
       </c>
       <c r="E77" s="12" t="n">
-        <v>131</v>
+        <v>161</v>
       </c>
       <c r="F77" s="13" t="n">
-        <v>92353332881</v>
+        <v>145779681118</v>
       </c>
       <c r="G77" s="12" t="n">
-        <v>131</v>
+        <v>161</v>
       </c>
       <c r="H77" s="13" t="n">
-        <v>63921201899.01</v>
+        <v>70786680805.01001</v>
       </c>
       <c r="I77" s="12" t="n">
-        <v>113</v>
+        <v>143</v>
       </c>
       <c r="J77" s="13" t="n">
-        <v>59472768099</v>
+        <v>66338247005</v>
       </c>
       <c r="K77" s="12" t="n">
-        <v>11</v>
+        <v>33</v>
       </c>
       <c r="L77" s="13" t="n">
-        <v>2478343628</v>
+        <v>4005987066</v>
       </c>
       <c r="M77" s="12" t="n">
         <v>78</v>
       </c>
       <c r="N77" s="13" t="n">
-        <v>36848397597</v>
+        <v>36853897597</v>
       </c>
     </row>
   </sheetData>
@@ -13093,13 +13051,13 @@
         <v>1</v>
       </c>
       <c r="D19" s="11" t="n">
-        <v>4988300000</v>
+        <v>5040000000</v>
       </c>
       <c r="E19" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F19" s="11" t="n">
-        <v>4988300000</v>
+        <v>5040000000</v>
       </c>
       <c r="G19" s="4" t="n">
         <v>1</v>
@@ -13143,45 +13101,29 @@
           <t>DINAS PERINDUSTRIAN, PERDAGANGAN, KOPERASI, USAHA KECIL DAN MENENGAH - 2.17.3.30.3.31.01.0000</t>
         </is>
       </c>
-      <c r="C20" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D20" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E20" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F20" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G20" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H20" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I20" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J20" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="C20" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D20" s="9" t="n">
+        <v>2688000000</v>
+      </c>
+      <c r="E20" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F20" s="9" t="n">
+        <v>2688000000</v>
+      </c>
+      <c r="G20" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="H20" s="9" t="n">
+        <v>2646500000</v>
+      </c>
+      <c r="I20" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="J20" s="9" t="n">
+        <v>2646500000</v>
       </c>
       <c r="K20" s="10" t="inlineStr">
         <is>
@@ -13564,40 +13506,28 @@
         </is>
       </c>
       <c r="C26" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="D26" s="9" t="n">
+        <v>5399320575</v>
+      </c>
+      <c r="E26" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="D26" s="9" t="n">
-        <v>2699320575</v>
-      </c>
-      <c r="E26" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F26" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G26" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H26" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I26" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J26" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="F26" s="9" t="n">
+        <v>2700000000</v>
+      </c>
+      <c r="G26" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="H26" s="9" t="n">
+        <v>2699298000</v>
+      </c>
+      <c r="I26" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="J26" s="9" t="n">
+        <v>2699298000</v>
       </c>
       <c r="K26" s="10" t="inlineStr">
         <is>
@@ -17040,28 +16970,28 @@
         </is>
       </c>
       <c r="C77" s="12" t="n">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="D77" s="13" t="n">
-        <v>273281535553</v>
+        <v>278721235553</v>
       </c>
       <c r="E77" s="12" t="n">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="F77" s="13" t="n">
-        <v>141675670800</v>
+        <v>147115370800</v>
       </c>
       <c r="G77" s="12" t="n">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="H77" s="13" t="n">
-        <v>65889582008.97</v>
+        <v>71235380008.97</v>
       </c>
       <c r="I77" s="12" t="n">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="J77" s="13" t="n">
-        <v>65889582008.97</v>
+        <v>71235380008.97</v>
       </c>
       <c r="K77" s="2" t="inlineStr">
         <is>

</xml_diff>